<commit_message>
📊 [auto] Economic data update — 2026-05-27 02:10 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-05-27.xlsx
+++ b/reports/excel/MacroPulse_2026-05-27.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>
@@ -59662,7 +59662,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-05-27 01:55 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 [auto] Economic data update — 2026-05-27 23:45 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-05-27.xlsx
+++ b/reports/excel/MacroPulse_2026-05-27.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2166,12 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>+0.020 pp</t>
+          <t>+0.080 pp</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>+0.090 pp</t>
+          <t>+0.200 pp</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -2228,12 +2228,12 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>4.32</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>+0.040 pp</t>
+          <t>+0.070 pp</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>+0.070 pp</t>
+          <t>+0.170 pp</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
@@ -2290,12 +2290,12 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>5.04</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>+0.200 pp</t>
+          <t>+0.140 pp</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>+0.060 pp</t>
+          <t>+0.130 pp</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -47930,47 +47930,47 @@
       </c>
       <c r="E120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.080 pp</t>
         </is>
       </c>
       <c r="G120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.200 pp</t>
         </is>
       </c>
       <c r="H120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="I120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.070 pp</t>
         </is>
       </c>
       <c r="J120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.170 pp</t>
         </is>
       </c>
       <c r="K120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>5.04</t>
         </is>
       </c>
       <c r="L120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.140 pp</t>
         </is>
       </c>
       <c r="M120" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+0.130 pp</t>
         </is>
       </c>
       <c r="N120" s="19" t="inlineStr">
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -59662,7 +59662,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-05-27 02:10 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-05-27 23:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>